<commit_message>
Update - correcion de scorings y normalaizacion de clases homologadas
</commit_message>
<xml_diff>
--- a/docs/A2_llave_class_uso/propuesta_homologacion.xlsx
+++ b/docs/A2_llave_class_uso/propuesta_homologacion.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jesus\Work\CR\Github\PGBM_actividad_1_diagnostico\docs\A2_llave_class_uso\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E681CCD-429D-448D-97F7-5A307D855C29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADECE595-AD79-4E2D-A0B3-B048A7A64C32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="leyenda_propuesta" sheetId="1" r:id="rId1"/>
-    <sheet name="homologacion" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet1" sheetId="3" r:id="rId3"/>
+    <sheet name="Propuesta_leyenda" sheetId="3" r:id="rId1"/>
+    <sheet name="leyenda_propuesta" sheetId="1" r:id="rId2"/>
+    <sheet name="homologacion" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
@@ -554,7 +554,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -570,7 +570,6 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -824,6 +823,1311 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5ADE2C7B-7B86-4289-92D6-0F937B4FDABD}">
+  <dimension ref="A1:J40"/>
+  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.33203125" customWidth="1"/>
+    <col min="2" max="2" width="31.77734375" customWidth="1"/>
+    <col min="3" max="3" width="11.33203125" customWidth="1"/>
+    <col min="4" max="4" width="45.44140625" customWidth="1"/>
+    <col min="5" max="5" width="11.33203125" customWidth="1"/>
+    <col min="6" max="6" width="59" customWidth="1"/>
+    <col min="7" max="7" width="15.88671875" customWidth="1"/>
+    <col min="8" max="8" width="31.77734375" customWidth="1"/>
+    <col min="9" max="9" width="15.88671875" customWidth="1"/>
+    <col min="10" max="10" width="38.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="8">
+        <v>40</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="C2" s="12">
+        <v>41</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="E2" s="12">
+        <v>410</v>
+      </c>
+      <c r="F2" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="G2" s="12">
+        <v>1</v>
+      </c>
+      <c r="H2" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="I2" s="12">
+        <v>11</v>
+      </c>
+      <c r="J2" s="12" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="8">
+        <v>40</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="C3" s="12">
+        <v>41</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="E3" s="12">
+        <v>411</v>
+      </c>
+      <c r="F3" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="G3" s="12">
+        <v>1</v>
+      </c>
+      <c r="H3" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="I3" s="12">
+        <v>11</v>
+      </c>
+      <c r="J3" s="12" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="8">
+        <v>40</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="C4" s="12">
+        <v>41</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="E4" s="12">
+        <v>412</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="G4" s="12">
+        <v>1</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="I4" s="12">
+        <v>11</v>
+      </c>
+      <c r="J4" s="12" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="8">
+        <v>40</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="C5" s="12">
+        <v>41</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="E5" s="12">
+        <v>413</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="G5" s="12">
+        <v>1</v>
+      </c>
+      <c r="H5" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="I5" s="12">
+        <v>11</v>
+      </c>
+      <c r="J5" s="12" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" s="8">
+        <v>40</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="C6" s="8">
+        <v>44</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="E6" s="8">
+        <v>441</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="G6" s="8">
+        <v>1</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="I6" s="8">
+        <v>11</v>
+      </c>
+      <c r="J6" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="8">
+        <v>40</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="C7" s="8">
+        <v>44</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="E7" s="8">
+        <v>444</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="G7" s="8">
+        <v>1</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="I7" s="8">
+        <v>11</v>
+      </c>
+      <c r="J7" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="8">
+        <v>40</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="C8" s="8">
+        <v>44</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="E8" s="8">
+        <v>445</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="G8" s="8">
+        <v>1</v>
+      </c>
+      <c r="H8" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="I8" s="8">
+        <v>11</v>
+      </c>
+      <c r="J8" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="8">
+        <v>40</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="C9" s="8">
+        <v>42</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="E9" s="8">
+        <v>420</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="G9" s="8">
+        <v>1</v>
+      </c>
+      <c r="H9" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="I9" s="8">
+        <v>12</v>
+      </c>
+      <c r="J9" s="8" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" s="8">
+        <v>40</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="C10" s="8">
+        <v>42</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="E10" s="8">
+        <v>421</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="G10" s="8">
+        <v>1</v>
+      </c>
+      <c r="H10" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="I10" s="8">
+        <v>12</v>
+      </c>
+      <c r="J10" s="8" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" s="8">
+        <v>40</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="C11" s="8">
+        <v>42</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="E11" s="8">
+        <v>422</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="G11" s="8">
+        <v>1</v>
+      </c>
+      <c r="H11" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="I11" s="8">
+        <v>12</v>
+      </c>
+      <c r="J11" s="8" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" s="8">
+        <v>40</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="C12" s="8">
+        <v>42</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="E12" s="8">
+        <v>423</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="G12" s="8">
+        <v>1</v>
+      </c>
+      <c r="H12" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="I12" s="8">
+        <v>12</v>
+      </c>
+      <c r="J12" s="8" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" s="8">
+        <v>40</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="C13" s="8">
+        <v>43</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="E13" s="8">
+        <v>430</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="G13" s="8">
+        <v>1</v>
+      </c>
+      <c r="H13" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="I13" s="8">
+        <v>13</v>
+      </c>
+      <c r="J13" s="8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" s="8">
+        <v>40</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="C14" s="8">
+        <v>43</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="E14" s="8">
+        <v>431</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="G14" s="8">
+        <v>1</v>
+      </c>
+      <c r="H14" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="I14" s="8">
+        <v>13</v>
+      </c>
+      <c r="J14" s="8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="8">
+        <v>40</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="C15" s="8">
+        <v>43</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="E15" s="8">
+        <v>432</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="G15" s="8">
+        <v>1</v>
+      </c>
+      <c r="H15" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="I15" s="8">
+        <v>13</v>
+      </c>
+      <c r="J15" s="8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" s="8">
+        <v>40</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="C16" s="13">
+        <v>41</v>
+      </c>
+      <c r="D16" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="E16" s="13">
+        <v>414</v>
+      </c>
+      <c r="F16" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="G16" s="13">
+        <v>1</v>
+      </c>
+      <c r="H16" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="I16" s="13">
+        <v>14</v>
+      </c>
+      <c r="J16" s="13" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" s="8">
+        <v>40</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="C17" s="8">
+        <v>44</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="E17" s="8">
+        <v>442</v>
+      </c>
+      <c r="F17" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="G17" s="8">
+        <v>1</v>
+      </c>
+      <c r="H17" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="I17" s="8">
+        <v>15</v>
+      </c>
+      <c r="J17" s="8" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A18" s="5">
+        <v>30</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C18" s="11">
+        <v>31</v>
+      </c>
+      <c r="D18" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="E18" s="11">
+        <v>311</v>
+      </c>
+      <c r="F18" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="G18" s="11">
+        <v>2</v>
+      </c>
+      <c r="H18" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="I18" s="11">
+        <v>21</v>
+      </c>
+      <c r="J18" s="11" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A19" s="5">
+        <v>30</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C19" s="5">
+        <v>32</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E19" s="5">
+        <v>321</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="G19" s="5">
+        <v>2</v>
+      </c>
+      <c r="H19" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I19" s="5">
+        <v>21</v>
+      </c>
+      <c r="J19" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A20" s="5">
+        <v>30</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C20" s="5">
+        <v>32</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E20" s="5">
+        <v>322</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="G20" s="5">
+        <v>2</v>
+      </c>
+      <c r="H20" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I20" s="5">
+        <v>21</v>
+      </c>
+      <c r="J20" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A21" s="5">
+        <v>30</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C21" s="5">
+        <v>32</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E21" s="5">
+        <v>323</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="G21" s="5">
+        <v>2</v>
+      </c>
+      <c r="H21" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I21" s="5">
+        <v>21</v>
+      </c>
+      <c r="J21" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A22" s="5">
+        <v>30</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C22" s="5">
+        <v>32</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E22" s="5">
+        <v>324</v>
+      </c>
+      <c r="F22" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="G22" s="5">
+        <v>2</v>
+      </c>
+      <c r="H22" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I22" s="5">
+        <v>21</v>
+      </c>
+      <c r="J22" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A23" s="7">
+        <v>30</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="C23" s="7">
+        <v>32</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="E23" s="7">
+        <v>325</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="G23" s="7">
+        <v>2</v>
+      </c>
+      <c r="H23" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="I23" s="7">
+        <v>21</v>
+      </c>
+      <c r="J23" s="7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A24" s="5">
+        <v>30</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C24" s="11">
+        <v>31</v>
+      </c>
+      <c r="D24" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="E24" s="11">
+        <v>312</v>
+      </c>
+      <c r="F24" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="G24" s="11">
+        <v>2</v>
+      </c>
+      <c r="H24" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="I24" s="11">
+        <v>22</v>
+      </c>
+      <c r="J24" s="11" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A25" s="5">
+        <v>30</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C25" s="11">
+        <v>31</v>
+      </c>
+      <c r="D25" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="E25" s="11">
+        <v>313</v>
+      </c>
+      <c r="F25" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="G25" s="11">
+        <v>2</v>
+      </c>
+      <c r="H25" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="I25" s="11">
+        <v>22</v>
+      </c>
+      <c r="J25" s="11" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A26" s="5">
+        <v>30</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C26" s="11">
+        <v>31</v>
+      </c>
+      <c r="D26" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="E26" s="11">
+        <v>314</v>
+      </c>
+      <c r="F26" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="G26" s="11">
+        <v>2</v>
+      </c>
+      <c r="H26" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="I26" s="11">
+        <v>22</v>
+      </c>
+      <c r="J26" s="11" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A27" s="5">
+        <v>30</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C27" s="11">
+        <v>31</v>
+      </c>
+      <c r="D27" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="E27" s="11">
+        <v>315</v>
+      </c>
+      <c r="F27" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="G27" s="11">
+        <v>2</v>
+      </c>
+      <c r="H27" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="I27" s="11">
+        <v>22</v>
+      </c>
+      <c r="J27" s="11" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A28" s="5">
+        <v>30</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C28" s="5">
+        <v>33</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="E28" s="5">
+        <v>331</v>
+      </c>
+      <c r="F28" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="G28" s="5">
+        <v>2</v>
+      </c>
+      <c r="H28" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I28" s="5">
+        <v>22</v>
+      </c>
+      <c r="J28" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A29" s="5">
+        <v>30</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C29" s="5">
+        <v>33</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="E29" s="5">
+        <v>332</v>
+      </c>
+      <c r="F29" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="G29" s="5">
+        <v>2</v>
+      </c>
+      <c r="H29" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I29" s="5">
+        <v>22</v>
+      </c>
+      <c r="J29" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A30" s="5">
+        <v>30</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C30" s="5">
+        <v>33</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="E30" s="5">
+        <v>333</v>
+      </c>
+      <c r="F30" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="G30" s="5">
+        <v>2</v>
+      </c>
+      <c r="H30" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I30" s="5">
+        <v>22</v>
+      </c>
+      <c r="J30" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A31" s="5">
+        <v>10</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C31" s="5">
+        <v>11</v>
+      </c>
+      <c r="D31" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E31" s="5">
+        <v>110</v>
+      </c>
+      <c r="F31" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G31" s="5">
+        <v>2</v>
+      </c>
+      <c r="H31" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I31" s="5">
+        <v>23</v>
+      </c>
+      <c r="J31" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A32" s="5">
+        <v>10</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C32" s="5">
+        <v>11</v>
+      </c>
+      <c r="D32" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E32" s="5">
+        <v>111</v>
+      </c>
+      <c r="F32" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="G32" s="5">
+        <v>2</v>
+      </c>
+      <c r="H32" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I32" s="5">
+        <v>23</v>
+      </c>
+      <c r="J32" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A33" s="5">
+        <v>10</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C33" s="5">
+        <v>11</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E33" s="5">
+        <v>112</v>
+      </c>
+      <c r="F33" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="G33" s="5">
+        <v>2</v>
+      </c>
+      <c r="H33" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I33" s="5">
+        <v>23</v>
+      </c>
+      <c r="J33" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A34" s="5">
+        <v>10</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C34" s="11">
+        <v>12</v>
+      </c>
+      <c r="D34" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="E34" s="11">
+        <v>121</v>
+      </c>
+      <c r="F34" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="G34" s="11">
+        <v>2</v>
+      </c>
+      <c r="H34" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="I34" s="11">
+        <v>23</v>
+      </c>
+      <c r="J34" s="11" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A35" s="5">
+        <v>20</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C35" s="5">
+        <v>21</v>
+      </c>
+      <c r="D35" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="E35" s="5">
+        <v>210</v>
+      </c>
+      <c r="F35" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="G35" s="5">
+        <v>2</v>
+      </c>
+      <c r="H35" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I35" s="5">
+        <v>24</v>
+      </c>
+      <c r="J35" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A36" s="5">
+        <v>20</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C36" s="5">
+        <v>21</v>
+      </c>
+      <c r="D36" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="E36" s="5">
+        <v>211</v>
+      </c>
+      <c r="F36" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="G36" s="5">
+        <v>2</v>
+      </c>
+      <c r="H36" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I36" s="5">
+        <v>24</v>
+      </c>
+      <c r="J36" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A37" s="5">
+        <v>20</v>
+      </c>
+      <c r="B37" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C37" s="5">
+        <v>21</v>
+      </c>
+      <c r="D37" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="E37" s="5">
+        <v>212</v>
+      </c>
+      <c r="F37" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G37" s="5">
+        <v>2</v>
+      </c>
+      <c r="H37" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I37" s="5">
+        <v>24</v>
+      </c>
+      <c r="J37" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A38" s="5">
+        <v>10</v>
+      </c>
+      <c r="B38" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C38" s="11">
+        <v>12</v>
+      </c>
+      <c r="D38" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="E38" s="11">
+        <v>122</v>
+      </c>
+      <c r="F38" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="G38" s="11">
+        <v>2</v>
+      </c>
+      <c r="H38" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="I38" s="11">
+        <v>25</v>
+      </c>
+      <c r="J38" s="11" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A39" s="6">
+        <v>20</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="C39" s="6">
+        <v>22</v>
+      </c>
+      <c r="D39" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E39" s="6">
+        <v>220</v>
+      </c>
+      <c r="F39" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="G39" s="6">
+        <v>2</v>
+      </c>
+      <c r="H39" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="I39" s="6">
+        <v>25</v>
+      </c>
+      <c r="J39" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A40" s="10">
+        <v>90</v>
+      </c>
+      <c r="B40" s="10" t="s">
+        <v>113</v>
+      </c>
+      <c r="C40" s="10">
+        <v>91</v>
+      </c>
+      <c r="D40" s="10" t="s">
+        <v>113</v>
+      </c>
+      <c r="E40" s="10">
+        <v>910</v>
+      </c>
+      <c r="F40" s="10" t="s">
+        <v>113</v>
+      </c>
+      <c r="G40" s="10">
+        <v>2</v>
+      </c>
+      <c r="H40" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="I40" s="10">
+        <v>25</v>
+      </c>
+      <c r="J40" s="10" t="s">
+        <v>20</v>
+      </c>
+    </row>
+  </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J42">
+    <sortCondition ref="I1:I42"/>
+  </sortState>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F12"/>
   <sheetFormatPr defaultColWidth="9.77734375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
@@ -832,7 +2136,7 @@
     <col min="2" max="2" width="31.77734375" customWidth="1"/>
     <col min="3" max="3" width="15.88671875" customWidth="1"/>
     <col min="4" max="4" width="38.5546875" customWidth="1"/>
-    <col min="5" max="5" width="68.109375" customWidth="1"/>
+    <col min="5" max="5" width="84" bestFit="1" customWidth="1"/>
     <col min="16383" max="16384" width="11.5546875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1041,7 +2345,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:M40"/>
   <sheetFormatPr defaultColWidth="9.77734375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
@@ -2509,1309 +3813,4 @@
     <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5ADE2C7B-7B86-4289-92D6-0F937B4FDABD}">
-  <dimension ref="A1:J40"/>
-  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="11.33203125" customWidth="1"/>
-    <col min="2" max="2" width="31.77734375" customWidth="1"/>
-    <col min="3" max="3" width="11.33203125" customWidth="1"/>
-    <col min="4" max="4" width="45.44140625" customWidth="1"/>
-    <col min="5" max="5" width="11.33203125" customWidth="1"/>
-    <col min="6" max="6" width="59" customWidth="1"/>
-    <col min="7" max="7" width="15.88671875" customWidth="1"/>
-    <col min="8" max="8" width="31.77734375" customWidth="1"/>
-    <col min="9" max="9" width="15.88671875" customWidth="1"/>
-    <col min="10" max="10" width="38.5546875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:10" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="8">
-        <v>40</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="C2" s="13">
-        <v>41</v>
-      </c>
-      <c r="D2" s="13" t="s">
-        <v>86</v>
-      </c>
-      <c r="E2" s="13">
-        <v>410</v>
-      </c>
-      <c r="F2" s="13" t="s">
-        <v>86</v>
-      </c>
-      <c r="G2" s="13">
-        <v>1</v>
-      </c>
-      <c r="H2" s="13" t="s">
-        <v>5</v>
-      </c>
-      <c r="I2" s="13">
-        <v>11</v>
-      </c>
-      <c r="J2" s="13" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="8">
-        <v>40</v>
-      </c>
-      <c r="B3" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="C3" s="13">
-        <v>41</v>
-      </c>
-      <c r="D3" s="13" t="s">
-        <v>86</v>
-      </c>
-      <c r="E3" s="13">
-        <v>411</v>
-      </c>
-      <c r="F3" s="13" t="s">
-        <v>90</v>
-      </c>
-      <c r="G3" s="13">
-        <v>1</v>
-      </c>
-      <c r="H3" s="13" t="s">
-        <v>5</v>
-      </c>
-      <c r="I3" s="13">
-        <v>11</v>
-      </c>
-      <c r="J3" s="13" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="8">
-        <v>40</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="C4" s="13">
-        <v>41</v>
-      </c>
-      <c r="D4" s="13" t="s">
-        <v>86</v>
-      </c>
-      <c r="E4" s="13">
-        <v>412</v>
-      </c>
-      <c r="F4" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="G4" s="13">
-        <v>1</v>
-      </c>
-      <c r="H4" s="13" t="s">
-        <v>5</v>
-      </c>
-      <c r="I4" s="13">
-        <v>11</v>
-      </c>
-      <c r="J4" s="13" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="8">
-        <v>40</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="C5" s="13">
-        <v>41</v>
-      </c>
-      <c r="D5" s="13" t="s">
-        <v>86</v>
-      </c>
-      <c r="E5" s="13">
-        <v>413</v>
-      </c>
-      <c r="F5" s="13" t="s">
-        <v>96</v>
-      </c>
-      <c r="G5" s="13">
-        <v>1</v>
-      </c>
-      <c r="H5" s="13" t="s">
-        <v>5</v>
-      </c>
-      <c r="I5" s="13">
-        <v>11</v>
-      </c>
-      <c r="J5" s="13" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" s="8">
-        <v>40</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="C6" s="8">
-        <v>44</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="E6" s="8">
-        <v>441</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>110</v>
-      </c>
-      <c r="G6" s="8">
-        <v>1</v>
-      </c>
-      <c r="H6" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="I6" s="8">
-        <v>11</v>
-      </c>
-      <c r="J6" s="9" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="8">
-        <v>40</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="C7" s="8">
-        <v>44</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="E7" s="8">
-        <v>444</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>111</v>
-      </c>
-      <c r="G7" s="8">
-        <v>1</v>
-      </c>
-      <c r="H7" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="I7" s="8">
-        <v>11</v>
-      </c>
-      <c r="J7" s="9" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8" s="8">
-        <v>40</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="C8" s="8">
-        <v>44</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="E8" s="8">
-        <v>445</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="G8" s="8">
-        <v>1</v>
-      </c>
-      <c r="H8" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="I8" s="8">
-        <v>11</v>
-      </c>
-      <c r="J8" s="9" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" s="8">
-        <v>40</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="C9" s="8">
-        <v>42</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="E9" s="8">
-        <v>420</v>
-      </c>
-      <c r="F9" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="G9" s="8">
-        <v>1</v>
-      </c>
-      <c r="H9" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="I9" s="8">
-        <v>12</v>
-      </c>
-      <c r="J9" s="8" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" s="8">
-        <v>40</v>
-      </c>
-      <c r="B10" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="C10" s="8">
-        <v>42</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="E10" s="8">
-        <v>421</v>
-      </c>
-      <c r="F10" s="8" t="s">
-        <v>102</v>
-      </c>
-      <c r="G10" s="8">
-        <v>1</v>
-      </c>
-      <c r="H10" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="I10" s="8">
-        <v>12</v>
-      </c>
-      <c r="J10" s="8" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11" s="8">
-        <v>40</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="C11" s="8">
-        <v>42</v>
-      </c>
-      <c r="D11" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="E11" s="8">
-        <v>422</v>
-      </c>
-      <c r="F11" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="G11" s="8">
-        <v>1</v>
-      </c>
-      <c r="H11" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="I11" s="8">
-        <v>12</v>
-      </c>
-      <c r="J11" s="8" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12" s="8">
-        <v>40</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="C12" s="8">
-        <v>42</v>
-      </c>
-      <c r="D12" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="E12" s="8">
-        <v>423</v>
-      </c>
-      <c r="F12" s="8" t="s">
-        <v>104</v>
-      </c>
-      <c r="G12" s="8">
-        <v>1</v>
-      </c>
-      <c r="H12" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="I12" s="8">
-        <v>12</v>
-      </c>
-      <c r="J12" s="8" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A13" s="8">
-        <v>40</v>
-      </c>
-      <c r="B13" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="C13" s="8">
-        <v>43</v>
-      </c>
-      <c r="D13" s="8" t="s">
-        <v>106</v>
-      </c>
-      <c r="E13" s="8">
-        <v>430</v>
-      </c>
-      <c r="F13" s="8" t="s">
-        <v>106</v>
-      </c>
-      <c r="G13" s="8">
-        <v>1</v>
-      </c>
-      <c r="H13" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="I13" s="8">
-        <v>13</v>
-      </c>
-      <c r="J13" s="8" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A14" s="8">
-        <v>40</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="C14" s="8">
-        <v>43</v>
-      </c>
-      <c r="D14" s="8" t="s">
-        <v>106</v>
-      </c>
-      <c r="E14" s="8">
-        <v>431</v>
-      </c>
-      <c r="F14" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="G14" s="8">
-        <v>1</v>
-      </c>
-      <c r="H14" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="I14" s="8">
-        <v>13</v>
-      </c>
-      <c r="J14" s="8" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A15" s="8">
-        <v>40</v>
-      </c>
-      <c r="B15" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="C15" s="8">
-        <v>43</v>
-      </c>
-      <c r="D15" s="8" t="s">
-        <v>106</v>
-      </c>
-      <c r="E15" s="8">
-        <v>432</v>
-      </c>
-      <c r="F15" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="G15" s="8">
-        <v>1</v>
-      </c>
-      <c r="H15" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="I15" s="8">
-        <v>13</v>
-      </c>
-      <c r="J15" s="8" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A16" s="8">
-        <v>40</v>
-      </c>
-      <c r="B16" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="C16" s="14">
-        <v>41</v>
-      </c>
-      <c r="D16" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="E16" s="14">
-        <v>414</v>
-      </c>
-      <c r="F16" s="14" t="s">
-        <v>98</v>
-      </c>
-      <c r="G16" s="14">
-        <v>1</v>
-      </c>
-      <c r="H16" s="14" t="s">
-        <v>5</v>
-      </c>
-      <c r="I16" s="14">
-        <v>14</v>
-      </c>
-      <c r="J16" s="14" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A17" s="8">
-        <v>40</v>
-      </c>
-      <c r="B17" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="C17" s="8">
-        <v>44</v>
-      </c>
-      <c r="D17" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="E17" s="8">
-        <v>442</v>
-      </c>
-      <c r="F17" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="G17" s="8">
-        <v>1</v>
-      </c>
-      <c r="H17" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="I17" s="8">
-        <v>15</v>
-      </c>
-      <c r="J17" s="8" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A18" s="5">
-        <v>30</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="C18" s="12">
-        <v>31</v>
-      </c>
-      <c r="D18" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="E18" s="12">
-        <v>311</v>
-      </c>
-      <c r="F18" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="G18" s="12">
-        <v>2</v>
-      </c>
-      <c r="H18" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="I18" s="12">
-        <v>21</v>
-      </c>
-      <c r="J18" s="12" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A19" s="5">
-        <v>30</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="C19" s="5">
-        <v>32</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="E19" s="5">
-        <v>321</v>
-      </c>
-      <c r="F19" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="G19" s="5">
-        <v>2</v>
-      </c>
-      <c r="H19" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="I19" s="5">
-        <v>21</v>
-      </c>
-      <c r="J19" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A20" s="5">
-        <v>30</v>
-      </c>
-      <c r="B20" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="C20" s="5">
-        <v>32</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="E20" s="5">
-        <v>322</v>
-      </c>
-      <c r="F20" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="G20" s="5">
-        <v>2</v>
-      </c>
-      <c r="H20" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="I20" s="5">
-        <v>21</v>
-      </c>
-      <c r="J20" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A21" s="5">
-        <v>30</v>
-      </c>
-      <c r="B21" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="C21" s="5">
-        <v>32</v>
-      </c>
-      <c r="D21" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="E21" s="5">
-        <v>323</v>
-      </c>
-      <c r="F21" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="G21" s="5">
-        <v>2</v>
-      </c>
-      <c r="H21" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="I21" s="5">
-        <v>21</v>
-      </c>
-      <c r="J21" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A22" s="5">
-        <v>30</v>
-      </c>
-      <c r="B22" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="C22" s="5">
-        <v>32</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="E22" s="5">
-        <v>324</v>
-      </c>
-      <c r="F22" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="G22" s="5">
-        <v>2</v>
-      </c>
-      <c r="H22" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="I22" s="5">
-        <v>21</v>
-      </c>
-      <c r="J22" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A23" s="7">
-        <v>30</v>
-      </c>
-      <c r="B23" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="C23" s="7">
-        <v>32</v>
-      </c>
-      <c r="D23" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="E23" s="7">
-        <v>325</v>
-      </c>
-      <c r="F23" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="G23" s="7">
-        <v>2</v>
-      </c>
-      <c r="H23" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="I23" s="7">
-        <v>21</v>
-      </c>
-      <c r="J23" s="7" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A24" s="5">
-        <v>30</v>
-      </c>
-      <c r="B24" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="C24" s="12">
-        <v>31</v>
-      </c>
-      <c r="D24" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="E24" s="12">
-        <v>312</v>
-      </c>
-      <c r="F24" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="G24" s="12">
-        <v>2</v>
-      </c>
-      <c r="H24" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="I24" s="12">
-        <v>22</v>
-      </c>
-      <c r="J24" s="12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A25" s="5">
-        <v>30</v>
-      </c>
-      <c r="B25" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="C25" s="12">
-        <v>31</v>
-      </c>
-      <c r="D25" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="E25" s="12">
-        <v>313</v>
-      </c>
-      <c r="F25" s="12" t="s">
-        <v>62</v>
-      </c>
-      <c r="G25" s="12">
-        <v>2</v>
-      </c>
-      <c r="H25" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="I25" s="12">
-        <v>22</v>
-      </c>
-      <c r="J25" s="12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A26" s="5">
-        <v>30</v>
-      </c>
-      <c r="B26" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="C26" s="12">
-        <v>31</v>
-      </c>
-      <c r="D26" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="E26" s="12">
-        <v>314</v>
-      </c>
-      <c r="F26" s="12" t="s">
-        <v>64</v>
-      </c>
-      <c r="G26" s="12">
-        <v>2</v>
-      </c>
-      <c r="H26" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="I26" s="12">
-        <v>22</v>
-      </c>
-      <c r="J26" s="12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A27" s="5">
-        <v>30</v>
-      </c>
-      <c r="B27" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="C27" s="12">
-        <v>31</v>
-      </c>
-      <c r="D27" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="E27" s="12">
-        <v>315</v>
-      </c>
-      <c r="F27" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="G27" s="12">
-        <v>2</v>
-      </c>
-      <c r="H27" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="I27" s="12">
-        <v>22</v>
-      </c>
-      <c r="J27" s="12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A28" s="5">
-        <v>30</v>
-      </c>
-      <c r="B28" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="C28" s="5">
-        <v>33</v>
-      </c>
-      <c r="D28" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="E28" s="5">
-        <v>331</v>
-      </c>
-      <c r="F28" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="G28" s="5">
-        <v>2</v>
-      </c>
-      <c r="H28" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="I28" s="5">
-        <v>22</v>
-      </c>
-      <c r="J28" s="5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A29" s="5">
-        <v>30</v>
-      </c>
-      <c r="B29" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="C29" s="5">
-        <v>33</v>
-      </c>
-      <c r="D29" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="E29" s="5">
-        <v>332</v>
-      </c>
-      <c r="F29" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="G29" s="5">
-        <v>2</v>
-      </c>
-      <c r="H29" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="I29" s="5">
-        <v>22</v>
-      </c>
-      <c r="J29" s="5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A30" s="11">
-        <v>30</v>
-      </c>
-      <c r="B30" s="11" t="s">
-        <v>56</v>
-      </c>
-      <c r="C30" s="11">
-        <v>33</v>
-      </c>
-      <c r="D30" s="11" t="s">
-        <v>76</v>
-      </c>
-      <c r="E30" s="11">
-        <v>333</v>
-      </c>
-      <c r="F30" s="11" t="s">
-        <v>82</v>
-      </c>
-      <c r="G30" s="11">
-        <v>2</v>
-      </c>
-      <c r="H30" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="I30" s="11">
-        <v>22</v>
-      </c>
-      <c r="J30" s="11" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A31" s="5">
-        <v>10</v>
-      </c>
-      <c r="B31" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="C31" s="5">
-        <v>11</v>
-      </c>
-      <c r="D31" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="E31" s="5">
-        <v>110</v>
-      </c>
-      <c r="F31" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="G31" s="5">
-        <v>2</v>
-      </c>
-      <c r="H31" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="I31" s="5">
-        <v>23</v>
-      </c>
-      <c r="J31" s="5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A32" s="5">
-        <v>10</v>
-      </c>
-      <c r="B32" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="C32" s="5">
-        <v>11</v>
-      </c>
-      <c r="D32" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="E32" s="5">
-        <v>111</v>
-      </c>
-      <c r="F32" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="G32" s="5">
-        <v>2</v>
-      </c>
-      <c r="H32" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="I32" s="5">
-        <v>23</v>
-      </c>
-      <c r="J32" s="5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A33" s="5">
-        <v>10</v>
-      </c>
-      <c r="B33" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="C33" s="5">
-        <v>11</v>
-      </c>
-      <c r="D33" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="E33" s="5">
-        <v>112</v>
-      </c>
-      <c r="F33" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="G33" s="5">
-        <v>2</v>
-      </c>
-      <c r="H33" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="I33" s="5">
-        <v>23</v>
-      </c>
-      <c r="J33" s="5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A34" s="5">
-        <v>10</v>
-      </c>
-      <c r="B34" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="C34" s="12">
-        <v>12</v>
-      </c>
-      <c r="D34" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="E34" s="12">
-        <v>121</v>
-      </c>
-      <c r="F34" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="G34" s="12">
-        <v>2</v>
-      </c>
-      <c r="H34" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="I34" s="12">
-        <v>23</v>
-      </c>
-      <c r="J34" s="12" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A35" s="5">
-        <v>20</v>
-      </c>
-      <c r="B35" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="C35" s="5">
-        <v>21</v>
-      </c>
-      <c r="D35" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="E35" s="5">
-        <v>210</v>
-      </c>
-      <c r="F35" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="G35" s="5">
-        <v>2</v>
-      </c>
-      <c r="H35" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="I35" s="5">
-        <v>24</v>
-      </c>
-      <c r="J35" s="5" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A36" s="5">
-        <v>20</v>
-      </c>
-      <c r="B36" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="C36" s="5">
-        <v>21</v>
-      </c>
-      <c r="D36" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="E36" s="5">
-        <v>211</v>
-      </c>
-      <c r="F36" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="G36" s="5">
-        <v>2</v>
-      </c>
-      <c r="H36" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="I36" s="5">
-        <v>24</v>
-      </c>
-      <c r="J36" s="5" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A37" s="5">
-        <v>20</v>
-      </c>
-      <c r="B37" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="C37" s="5">
-        <v>21</v>
-      </c>
-      <c r="D37" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="E37" s="5">
-        <v>212</v>
-      </c>
-      <c r="F37" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="G37" s="5">
-        <v>2</v>
-      </c>
-      <c r="H37" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="I37" s="5">
-        <v>24</v>
-      </c>
-      <c r="J37" s="5" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A38" s="5">
-        <v>10</v>
-      </c>
-      <c r="B38" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="C38" s="12">
-        <v>12</v>
-      </c>
-      <c r="D38" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="E38" s="12">
-        <v>122</v>
-      </c>
-      <c r="F38" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="G38" s="12">
-        <v>2</v>
-      </c>
-      <c r="H38" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="I38" s="12">
-        <v>25</v>
-      </c>
-      <c r="J38" s="12" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A39" s="6">
-        <v>20</v>
-      </c>
-      <c r="B39" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="C39" s="6">
-        <v>22</v>
-      </c>
-      <c r="D39" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="E39" s="6">
-        <v>220</v>
-      </c>
-      <c r="F39" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="G39" s="6">
-        <v>2</v>
-      </c>
-      <c r="H39" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="I39" s="6">
-        <v>25</v>
-      </c>
-      <c r="J39" s="6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A40" s="10">
-        <v>90</v>
-      </c>
-      <c r="B40" s="10" t="s">
-        <v>113</v>
-      </c>
-      <c r="C40" s="10">
-        <v>91</v>
-      </c>
-      <c r="D40" s="10" t="s">
-        <v>113</v>
-      </c>
-      <c r="E40" s="10">
-        <v>910</v>
-      </c>
-      <c r="F40" s="10" t="s">
-        <v>113</v>
-      </c>
-      <c r="G40" s="10">
-        <v>2</v>
-      </c>
-      <c r="H40" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="I40" s="10">
-        <v>25</v>
-      </c>
-      <c r="J40" s="10" t="s">
-        <v>20</v>
-      </c>
-    </row>
-  </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J42">
-    <sortCondition ref="I1:I42"/>
-  </sortState>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>